<commit_message>
Tree Years is misbehaving
</commit_message>
<xml_diff>
--- a/Source/Tech Tree/Tree Years.xlsx
+++ b/Source/Tech Tree/Tree Years.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/53f841be2cb91021/Desktop/KSP Mods/RP-1_Crow/Source/Tech Tree/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{01127C48-2EE7-4688-98D4-1807BF7743F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5459B88C-B166-5DAB-983A-B71C1D7EF2CB}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{01127C48-2EE7-4688-98D4-1807BF7743F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97F83FEB-A72D-481E-BA6F-40D1394FC629}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{73CA1BD0-04E5-4D1A-9F47-B0D01E7997A1}"/>
   </bookViews>
@@ -1108,7 +1108,8 @@
   <autoFilter ref="A1:C1963" xr:uid="{9BA48B2D-B23C-4546-9267-C4BE6CED0FC8}">
     <filterColumn colId="2">
       <filters>
-        <filter val="Comms"/>
+        <filter val="Spaceplanes"/>
+        <filter val="Stations"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -9245,7 +9246,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="108" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A108">
         <v>0</v>
       </c>
@@ -9256,7 +9257,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="109" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A109">
         <v>1950</v>
       </c>
@@ -9267,7 +9268,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="110" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A110">
         <v>1951</v>
       </c>
@@ -9278,7 +9279,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="111" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A111">
         <v>1952</v>
       </c>
@@ -9289,7 +9290,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="112" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A112">
         <v>1953</v>
       </c>
@@ -9300,7 +9301,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="113" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A113">
         <v>1954</v>
       </c>
@@ -9311,7 +9312,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="114" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A114">
         <v>1955</v>
       </c>
@@ -9322,7 +9323,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="115" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A115">
         <v>1956</v>
       </c>
@@ -9333,7 +9334,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="116" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A116">
         <v>1957</v>
       </c>
@@ -9344,7 +9345,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="117" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A117">
         <v>1958</v>
       </c>
@@ -9355,7 +9356,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="118" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>1959</v>
       </c>
@@ -9366,7 +9367,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="119" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>1960</v>
       </c>
@@ -9377,7 +9378,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="120" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A120">
         <v>1961</v>
       </c>
@@ -9388,7 +9389,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="121" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A121">
         <v>1962</v>
       </c>
@@ -9399,7 +9400,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="122" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A122">
         <v>1963</v>
       </c>
@@ -9410,7 +9411,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="123" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A123">
         <v>1964</v>
       </c>
@@ -9421,7 +9422,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="124" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A124">
         <v>1965</v>
       </c>
@@ -9432,7 +9433,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="125" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A125">
         <v>1966</v>
       </c>
@@ -9443,7 +9444,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="126" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A126">
         <v>1967</v>
       </c>
@@ -9454,7 +9455,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="127" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A127">
         <v>1968</v>
       </c>
@@ -9465,7 +9466,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="128" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A128">
         <v>1969</v>
       </c>
@@ -9476,7 +9477,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="129" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A129">
         <v>1970</v>
       </c>
@@ -9487,7 +9488,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="130" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A130">
         <v>1971</v>
       </c>
@@ -9498,7 +9499,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="131" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A131">
         <v>1972</v>
       </c>
@@ -9509,7 +9510,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="132" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A132">
         <v>1973</v>
       </c>
@@ -9520,7 +9521,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="133" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A133">
         <v>1974</v>
       </c>
@@ -9531,7 +9532,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="134" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A134">
         <v>1975</v>
       </c>
@@ -9542,7 +9543,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="135" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A135">
         <v>1976</v>
       </c>
@@ -9553,7 +9554,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="136" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A136">
         <v>1977</v>
       </c>
@@ -9564,7 +9565,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="137" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A137">
         <v>1978</v>
       </c>
@@ -9575,7 +9576,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="138" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A138">
         <v>1979</v>
       </c>
@@ -9586,7 +9587,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="139" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A139">
         <v>1980</v>
       </c>
@@ -9597,7 +9598,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="140" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A140">
         <v>1981</v>
       </c>
@@ -9608,7 +9609,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="141" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A141">
         <v>1982</v>
       </c>
@@ -9619,7 +9620,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="142" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A142">
         <v>1983</v>
       </c>
@@ -9630,7 +9631,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="143" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A143">
         <v>1984</v>
       </c>
@@ -9641,7 +9642,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="144" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A144">
         <v>1985</v>
       </c>
@@ -9652,7 +9653,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="145" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A145">
         <v>1986</v>
       </c>
@@ -9663,7 +9664,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="146" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A146">
         <v>1987</v>
       </c>
@@ -9674,7 +9675,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="147" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A147">
         <v>1988</v>
       </c>
@@ -9685,7 +9686,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="148" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A148">
         <v>1989</v>
       </c>
@@ -9696,7 +9697,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="149" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A149">
         <v>1990</v>
       </c>
@@ -9707,7 +9708,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="150" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A150">
         <v>1991</v>
       </c>
@@ -9718,7 +9719,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="151" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A151">
         <v>1992</v>
       </c>
@@ -9729,7 +9730,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="152" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A152">
         <v>1993</v>
       </c>
@@ -9740,7 +9741,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="153" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A153">
         <v>1994</v>
       </c>
@@ -9751,7 +9752,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="154" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A154">
         <v>1995</v>
       </c>
@@ -9762,7 +9763,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="155" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A155">
         <v>1996</v>
       </c>
@@ -9773,7 +9774,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="156" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A156">
         <v>1997</v>
       </c>
@@ -9784,7 +9785,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="157" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A157">
         <v>1998</v>
       </c>
@@ -9795,7 +9796,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="158" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A158">
         <v>1999</v>
       </c>
@@ -9806,7 +9807,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="159" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A159">
         <v>2000</v>
       </c>
@@ -9817,7 +9818,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="160" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A160">
         <v>2001</v>
       </c>
@@ -9828,7 +9829,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="161" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A161">
         <v>2002</v>
       </c>
@@ -9839,7 +9840,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="162" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A162">
         <v>2003</v>
       </c>
@@ -9850,7 +9851,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="163" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A163">
         <v>2004</v>
       </c>
@@ -9861,7 +9862,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="164" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A164">
         <v>2005</v>
       </c>
@@ -9872,7 +9873,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="165" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A165">
         <v>2006</v>
       </c>
@@ -9883,7 +9884,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="166" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A166">
         <v>2007</v>
       </c>
@@ -9894,7 +9895,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="167" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A167">
         <v>2008</v>
       </c>
@@ -9905,7 +9906,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="168" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A168">
         <v>2009</v>
       </c>
@@ -9916,7 +9917,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="169" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A169">
         <v>2010</v>
       </c>
@@ -9927,7 +9928,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="170" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A170">
         <v>2011</v>
       </c>
@@ -9938,7 +9939,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="171" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A171">
         <v>2012</v>
       </c>
@@ -9949,7 +9950,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="172" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A172">
         <v>2013</v>
       </c>
@@ -9960,7 +9961,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="173" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A173">
         <v>2014</v>
       </c>
@@ -9971,7 +9972,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="174" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A174">
         <v>2015</v>
       </c>
@@ -9982,7 +9983,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="175" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A175">
         <v>2016</v>
       </c>
@@ -9993,7 +9994,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="176" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A176">
         <v>2017</v>
       </c>
@@ -10004,7 +10005,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="177" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A177">
         <v>2018</v>
       </c>
@@ -10015,7 +10016,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="178" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A178">
         <v>2019</v>
       </c>
@@ -10026,7 +10027,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="179" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A179">
         <v>2020</v>
       </c>
@@ -10037,7 +10038,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="180" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A180">
         <v>2021</v>
       </c>
@@ -10048,7 +10049,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="181" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A181">
         <v>2022</v>
       </c>
@@ -10059,7 +10060,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="182" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A182">
         <v>2023</v>
       </c>
@@ -10070,7 +10071,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="183" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A183">
         <v>2024</v>
       </c>
@@ -10081,7 +10082,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="184" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A184">
         <v>2025</v>
       </c>
@@ -10092,7 +10093,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="185" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A185">
         <v>2026</v>
       </c>
@@ -10103,7 +10104,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="186" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A186">
         <v>2027</v>
       </c>
@@ -10114,7 +10115,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="187" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A187">
         <v>2028</v>
       </c>
@@ -10125,7 +10126,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="188" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A188">
         <v>2029</v>
       </c>
@@ -10136,7 +10137,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="189" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A189">
         <v>2030</v>
       </c>
@@ -10147,7 +10148,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="190" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A190">
         <v>2031</v>
       </c>
@@ -10158,7 +10159,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="191" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A191">
         <v>2032</v>
       </c>
@@ -10169,7 +10170,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="192" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A192">
         <v>2033</v>
       </c>
@@ -10180,7 +10181,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="193" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A193">
         <v>2034</v>
       </c>
@@ -10191,7 +10192,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="194" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A194">
         <v>2035</v>
       </c>
@@ -10202,7 +10203,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="195" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A195">
         <v>2036</v>
       </c>
@@ -10213,7 +10214,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="196" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A196">
         <v>2037</v>
       </c>
@@ -10224,7 +10225,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="197" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A197">
         <v>2038</v>
       </c>
@@ -10235,7 +10236,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="198" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A198">
         <v>2039</v>
       </c>
@@ -10246,7 +10247,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="199" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A199">
         <v>2040</v>
       </c>
@@ -10257,7 +10258,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="200" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A200">
         <v>2041</v>
       </c>
@@ -10268,7 +10269,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="201" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A201">
         <v>2042</v>
       </c>
@@ -10279,7 +10280,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="202" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A202">
         <v>2043</v>
       </c>
@@ -10290,7 +10291,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="203" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A203">
         <v>2044</v>
       </c>
@@ -10301,7 +10302,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="204" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A204">
         <v>2045</v>
       </c>
@@ -10312,7 +10313,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="205" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A205">
         <v>2046</v>
       </c>
@@ -10323,7 +10324,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="206" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A206">
         <v>2047</v>
       </c>
@@ -10334,7 +10335,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="207" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A207">
         <v>2048</v>
       </c>
@@ -10345,7 +10346,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="208" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A208">
         <v>2049</v>
       </c>
@@ -10356,7 +10357,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="209" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A209">
         <v>2050</v>
       </c>
@@ -10367,7 +10368,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="210" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A210">
         <v>2051</v>
       </c>
@@ -10378,7 +10379,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="211" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A211">
         <v>2100</v>
       </c>
@@ -10389,7 +10390,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="212" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A212">
         <v>2150</v>
       </c>
@@ -10400,7 +10401,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="213" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
         <v>1</v>
       </c>
@@ -11445,7 +11446,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="308" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A308">
         <v>0</v>
       </c>
@@ -11456,7 +11457,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="309" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A309">
         <v>1967</v>
       </c>
@@ -11467,7 +11468,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="310" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A310">
         <v>1968</v>
       </c>
@@ -11478,7 +11479,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="311" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A311">
         <v>1969</v>
       </c>
@@ -11489,7 +11490,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="312" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A312">
         <v>1970</v>
       </c>
@@ -11500,7 +11501,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="313" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A313">
         <v>1971</v>
       </c>
@@ -11511,7 +11512,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="314" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A314">
         <v>1972</v>
       </c>
@@ -11522,7 +11523,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="315" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A315">
         <v>1973</v>
       </c>
@@ -11533,7 +11534,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="316" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A316">
         <v>1974</v>
       </c>
@@ -11544,7 +11545,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="317" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A317">
         <v>1975</v>
       </c>
@@ -11555,7 +11556,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="318" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A318">
         <v>1976</v>
       </c>
@@ -11566,7 +11567,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="319" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A319">
         <v>1977</v>
       </c>
@@ -11577,7 +11578,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="320" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A320">
         <v>1978</v>
       </c>
@@ -11588,7 +11589,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="321" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A321">
         <v>1979</v>
       </c>
@@ -11599,7 +11600,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="322" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A322">
         <v>1980</v>
       </c>
@@ -11610,7 +11611,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="323" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A323">
         <v>1981</v>
       </c>
@@ -11621,7 +11622,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="324" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A324">
         <v>1982</v>
       </c>
@@ -11632,7 +11633,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="325" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A325">
         <v>1983</v>
       </c>
@@ -11643,7 +11644,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="326" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A326">
         <v>1984</v>
       </c>
@@ -11654,7 +11655,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="327" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A327">
         <v>1985</v>
       </c>
@@ -11665,7 +11666,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="328" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A328">
         <v>1986</v>
       </c>
@@ -11676,7 +11677,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="329" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A329">
         <v>1987</v>
       </c>
@@ -11687,7 +11688,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="330" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A330">
         <v>1988</v>
       </c>
@@ -11698,7 +11699,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="331" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A331">
         <v>1989</v>
       </c>
@@ -11709,7 +11710,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="332" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A332">
         <v>1990</v>
       </c>
@@ -11720,7 +11721,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="333" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A333">
         <v>1991</v>
       </c>
@@ -11731,7 +11732,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="334" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A334">
         <v>1992</v>
       </c>
@@ -11742,7 +11743,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="335" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A335">
         <v>1993</v>
       </c>
@@ -11753,7 +11754,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="336" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A336">
         <v>1994</v>
       </c>
@@ -11764,7 +11765,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="337" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A337">
         <v>1995</v>
       </c>
@@ -11775,7 +11776,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="338" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A338">
         <v>1996</v>
       </c>
@@ -11786,7 +11787,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="339" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A339">
         <v>1997</v>
       </c>
@@ -11797,7 +11798,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="340" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A340">
         <v>1998</v>
       </c>
@@ -11808,7 +11809,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="341" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A341">
         <v>1999</v>
       </c>
@@ -11819,7 +11820,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="342" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A342">
         <v>2000</v>
       </c>
@@ -11830,7 +11831,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="343" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A343">
         <v>2001</v>
       </c>
@@ -11841,7 +11842,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="344" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A344">
         <v>2002</v>
       </c>
@@ -11852,7 +11853,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="345" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A345">
         <v>2003</v>
       </c>
@@ -11863,7 +11864,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="346" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A346">
         <v>2004</v>
       </c>
@@ -11874,7 +11875,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="347" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A347">
         <v>2005</v>
       </c>
@@ -11885,7 +11886,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="348" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A348">
         <v>2006</v>
       </c>
@@ -11896,7 +11897,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="349" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A349">
         <v>2007</v>
       </c>
@@ -11907,7 +11908,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="350" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A350">
         <v>2008</v>
       </c>
@@ -11918,7 +11919,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="351" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A351">
         <v>2009</v>
       </c>
@@ -11929,7 +11930,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="352" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A352">
         <v>2010</v>
       </c>
@@ -11940,7 +11941,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="353" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A353">
         <v>2011</v>
       </c>
@@ -11951,7 +11952,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="354" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A354">
         <v>2012</v>
       </c>
@@ -11962,7 +11963,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="355" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A355">
         <v>2013</v>
       </c>
@@ -11973,7 +11974,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="356" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A356">
         <v>2014</v>
       </c>
@@ -11984,7 +11985,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="357" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A357">
         <v>2015</v>
       </c>
@@ -11995,7 +11996,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="358" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A358">
         <v>2016</v>
       </c>
@@ -12006,7 +12007,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="359" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A359">
         <v>2017</v>
       </c>
@@ -12017,7 +12018,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="360" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A360">
         <v>2018</v>
       </c>
@@ -12028,7 +12029,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="361" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A361">
         <v>2019</v>
       </c>
@@ -12039,7 +12040,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="362" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A362">
         <v>2020</v>
       </c>
@@ -12050,7 +12051,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="363" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A363">
         <v>2021</v>
       </c>
@@ -12061,7 +12062,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="364" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A364">
         <v>2022</v>
       </c>
@@ -12072,7 +12073,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="365" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A365">
         <v>2023</v>
       </c>
@@ -12083,7 +12084,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="366" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A366">
         <v>2024</v>
       </c>
@@ -12094,7 +12095,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="367" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A367">
         <v>2025</v>
       </c>
@@ -12105,7 +12106,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="368" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A368">
         <v>2026</v>
       </c>
@@ -12116,7 +12117,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="369" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A369">
         <v>2027</v>
       </c>
@@ -12127,7 +12128,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="370" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A370">
         <v>2028</v>
       </c>
@@ -12138,7 +12139,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="371" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A371">
         <v>2029</v>
       </c>
@@ -12149,7 +12150,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="372" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A372">
         <v>2030</v>
       </c>
@@ -12160,7 +12161,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="373" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A373">
         <v>2031</v>
       </c>
@@ -12171,7 +12172,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="374" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A374">
         <v>2032</v>
       </c>
@@ -12182,7 +12183,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="375" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A375">
         <v>2033</v>
       </c>
@@ -12193,7 +12194,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="376" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A376">
         <v>2034</v>
       </c>
@@ -12204,7 +12205,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="377" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A377">
         <v>2035</v>
       </c>
@@ -12215,7 +12216,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="378" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A378">
         <v>2036</v>
       </c>
@@ -12226,7 +12227,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="379" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A379">
         <v>2037</v>
       </c>
@@ -12237,7 +12238,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="380" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A380">
         <v>2038</v>
       </c>
@@ -12248,7 +12249,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="381" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A381">
         <v>2039</v>
       </c>
@@ -12259,7 +12260,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="382" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A382">
         <v>2040</v>
       </c>
@@ -12270,7 +12271,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="383" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="383" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A383">
         <v>2041</v>
       </c>
@@ -12281,7 +12282,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="384" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="384" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A384">
         <v>2042</v>
       </c>
@@ -12292,7 +12293,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="385" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="385" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A385">
         <v>2043</v>
       </c>
@@ -12303,7 +12304,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="386" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="386" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A386">
         <v>2044</v>
       </c>
@@ -12314,7 +12315,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="387" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="387" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A387">
         <v>2045</v>
       </c>
@@ -12325,7 +12326,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="388" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="388" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A388">
         <v>2046</v>
       </c>
@@ -12336,7 +12337,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="389" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="389" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A389">
         <v>2047</v>
       </c>
@@ -12347,7 +12348,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="390" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="390" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A390">
         <v>2048</v>
       </c>
@@ -12358,7 +12359,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="391" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="391" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A391">
         <v>2049</v>
       </c>
@@ -12369,7 +12370,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="392" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="392" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A392">
         <v>2050</v>
       </c>
@@ -12380,7 +12381,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="393" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="393" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A393">
         <v>2051</v>
       </c>
@@ -12391,7 +12392,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="394" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="394" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A394">
         <v>2100</v>
       </c>
@@ -12402,7 +12403,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="395" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="395" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A395">
         <v>2150</v>
       </c>
@@ -26240,7 +26241,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="1653" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1653" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1653">
         <v>0</v>
       </c>
@@ -26251,7 +26252,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1654" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1654" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1654">
         <v>1956</v>
       </c>
@@ -26262,7 +26263,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1655" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1655" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1655">
         <v>1957</v>
       </c>
@@ -26273,7 +26274,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1656" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1656" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1656">
         <v>1958</v>
       </c>
@@ -26284,7 +26285,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1657" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1657" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1657">
         <v>1959</v>
       </c>
@@ -26295,7 +26296,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1658" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1658" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1658">
         <v>1960</v>
       </c>
@@ -26306,7 +26307,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1659" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1659" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1659">
         <v>1961</v>
       </c>
@@ -26317,7 +26318,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1660" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1660" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1660">
         <v>1962</v>
       </c>
@@ -26328,7 +26329,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1661" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1661" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1661">
         <v>1963</v>
       </c>
@@ -26339,7 +26340,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1662" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1662" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1662">
         <v>1964</v>
       </c>
@@ -26350,7 +26351,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1663" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1663" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1663">
         <v>1965</v>
       </c>
@@ -26361,7 +26362,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1664" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1664" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1664">
         <v>1966</v>
       </c>
@@ -26372,7 +26373,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1665" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1665" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1665">
         <v>1967</v>
       </c>
@@ -26383,7 +26384,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1666" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1666" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1666">
         <v>1968</v>
       </c>
@@ -26394,7 +26395,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1667" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1667" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1667">
         <v>1969</v>
       </c>
@@ -26405,7 +26406,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1668" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1668" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1668">
         <v>1970</v>
       </c>
@@ -26416,7 +26417,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1669" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1669" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1669">
         <v>1971</v>
       </c>
@@ -26427,7 +26428,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1670" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1670" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1670">
         <v>1972</v>
       </c>
@@ -26438,7 +26439,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1671" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1671" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1671">
         <v>1973</v>
       </c>
@@ -26449,7 +26450,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1672" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1672" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1672">
         <v>1974</v>
       </c>
@@ -26460,7 +26461,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1673" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1673" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1673">
         <v>1975</v>
       </c>
@@ -26471,7 +26472,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1674" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1674" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1674">
         <v>1976</v>
       </c>
@@ -26482,7 +26483,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1675" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1675" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1675">
         <v>1977</v>
       </c>
@@ -26493,7 +26494,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1676" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1676" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1676">
         <v>1978</v>
       </c>
@@ -26504,7 +26505,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1677" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1677" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1677">
         <v>1979</v>
       </c>
@@ -26515,7 +26516,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1678" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1678" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1678">
         <v>1980</v>
       </c>
@@ -26526,7 +26527,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1679" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1679" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1679">
         <v>1981</v>
       </c>
@@ -26537,7 +26538,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1680" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1680" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1680">
         <v>1982</v>
       </c>
@@ -26548,7 +26549,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1681" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1681" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1681">
         <v>1983</v>
       </c>
@@ -26559,7 +26560,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1682" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1682" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1682">
         <v>1984</v>
       </c>
@@ -26570,7 +26571,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1683" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1683" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1683">
         <v>1985</v>
       </c>
@@ -26581,7 +26582,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1684" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1684" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1684">
         <v>1986</v>
       </c>
@@ -26592,7 +26593,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1685" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1685" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1685">
         <v>1987</v>
       </c>
@@ -26603,7 +26604,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1686" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1686" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1686">
         <v>1988</v>
       </c>
@@ -26614,7 +26615,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1687" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1687" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1687">
         <v>1989</v>
       </c>
@@ -26625,7 +26626,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1688" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1688" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1688">
         <v>1990</v>
       </c>
@@ -26636,7 +26637,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1689" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1689" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1689">
         <v>1991</v>
       </c>
@@ -26647,7 +26648,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1690" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1690" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1690">
         <v>1992</v>
       </c>
@@ -26658,7 +26659,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1691" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1691" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1691">
         <v>1993</v>
       </c>
@@ -26669,7 +26670,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1692" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1692" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1692">
         <v>1994</v>
       </c>
@@ -26680,7 +26681,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1693" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1693" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1693">
         <v>1995</v>
       </c>
@@ -26691,7 +26692,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1694" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1694" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1694">
         <v>1996</v>
       </c>
@@ -26702,7 +26703,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1695" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1695" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1695">
         <v>1997</v>
       </c>
@@ -26713,7 +26714,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1696" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1696" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1696">
         <v>1998</v>
       </c>
@@ -26724,7 +26725,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1697" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1697" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1697">
         <v>1999</v>
       </c>
@@ -26735,7 +26736,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1698" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1698" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1698">
         <v>2000</v>
       </c>
@@ -26746,7 +26747,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1699" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1699" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1699">
         <v>2001</v>
       </c>
@@ -26757,7 +26758,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1700" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1700" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1700">
         <v>2002</v>
       </c>
@@ -26768,7 +26769,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1701" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1701" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1701">
         <v>2003</v>
       </c>
@@ -26779,7 +26780,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1702" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1702" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1702">
         <v>2004</v>
       </c>
@@ -26790,7 +26791,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1703" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1703" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1703">
         <v>2005</v>
       </c>
@@ -26801,7 +26802,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1704" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1704" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1704">
         <v>2006</v>
       </c>
@@ -26812,7 +26813,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1705" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1705" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1705">
         <v>2007</v>
       </c>
@@ -26823,7 +26824,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1706" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1706" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1706">
         <v>2008</v>
       </c>
@@ -26834,7 +26835,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1707" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1707" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1707">
         <v>2009</v>
       </c>
@@ -26845,7 +26846,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1708" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1708" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1708">
         <v>2010</v>
       </c>
@@ -26856,7 +26857,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1709" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1709" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1709">
         <v>2011</v>
       </c>
@@ -26867,7 +26868,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1710" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1710" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1710">
         <v>2012</v>
       </c>
@@ -26878,7 +26879,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1711" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1711" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1711">
         <v>2013</v>
       </c>
@@ -26889,7 +26890,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1712" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1712" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1712">
         <v>2014</v>
       </c>
@@ -26900,7 +26901,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1713" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1713" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1713">
         <v>2015</v>
       </c>
@@ -26911,7 +26912,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1714" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1714" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1714">
         <v>2016</v>
       </c>
@@ -26922,7 +26923,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1715" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1715" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1715">
         <v>2017</v>
       </c>
@@ -26933,7 +26934,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1716" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1716" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1716">
         <v>2018</v>
       </c>
@@ -26944,7 +26945,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1717" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1717" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1717">
         <v>2019</v>
       </c>
@@ -26955,7 +26956,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1718" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1718" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1718">
         <v>2020</v>
       </c>
@@ -26966,7 +26967,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1719" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1719" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1719">
         <v>2021</v>
       </c>
@@ -26977,7 +26978,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1720" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1720" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1720">
         <v>2022</v>
       </c>
@@ -26988,7 +26989,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1721" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1721" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1721">
         <v>2023</v>
       </c>
@@ -26999,7 +27000,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1722" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1722" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1722">
         <v>2024</v>
       </c>
@@ -27010,7 +27011,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1723" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1723" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1723">
         <v>2025</v>
       </c>
@@ -27021,7 +27022,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1724" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1724" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1724">
         <v>2026</v>
       </c>
@@ -27032,7 +27033,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1725" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1725" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1725">
         <v>2027</v>
       </c>
@@ -27043,7 +27044,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1726" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1726" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1726">
         <v>2028</v>
       </c>
@@ -27054,7 +27055,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1727" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1727" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1727">
         <v>2029</v>
       </c>
@@ -27065,7 +27066,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1728" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1728" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1728">
         <v>2030</v>
       </c>
@@ -27076,7 +27077,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1729" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1729" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1729">
         <v>2031</v>
       </c>
@@ -27087,7 +27088,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1730" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1730" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1730">
         <v>2032</v>
       </c>
@@ -27098,7 +27099,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1731" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1731" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1731">
         <v>2033</v>
       </c>
@@ -27109,7 +27110,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1732" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1732" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1732">
         <v>2034</v>
       </c>
@@ -27120,7 +27121,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1733" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1733" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1733">
         <v>2035</v>
       </c>
@@ -27131,7 +27132,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1734" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1734" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1734">
         <v>2036</v>
       </c>
@@ -27142,7 +27143,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1735" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1735" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1735">
         <v>2037</v>
       </c>
@@ -27153,7 +27154,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1736" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1736" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1736">
         <v>2038</v>
       </c>
@@ -27164,7 +27165,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1737" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1737" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1737">
         <v>2039</v>
       </c>
@@ -27175,7 +27176,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1738" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1738" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1738">
         <v>2040</v>
       </c>
@@ -27186,7 +27187,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1739" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1739" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1739">
         <v>2041</v>
       </c>
@@ -27197,7 +27198,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1740" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1740" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1740">
         <v>2042</v>
       </c>
@@ -27208,7 +27209,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1741" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1741" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1741">
         <v>2043</v>
       </c>
@@ -27219,7 +27220,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1742" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1742" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1742">
         <v>2044</v>
       </c>
@@ -27230,7 +27231,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1743" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1743" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1743">
         <v>2045</v>
       </c>
@@ -27241,7 +27242,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1744" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1744" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1744">
         <v>2046</v>
       </c>
@@ -27252,7 +27253,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1745" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1745" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1745">
         <v>2047</v>
       </c>
@@ -27263,7 +27264,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1746" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1746" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1746">
         <v>2048</v>
       </c>
@@ -27274,7 +27275,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1747" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1747" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1747">
         <v>2049</v>
       </c>
@@ -27285,7 +27286,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1748" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1748" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1748">
         <v>2050</v>
       </c>
@@ -27296,7 +27297,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1749" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1749" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1749">
         <v>2051</v>
       </c>
@@ -27307,7 +27308,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1750" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1750" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1750">
         <v>2100</v>
       </c>
@@ -27318,7 +27319,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="1751" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1751" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1751">
         <v>2150</v>
       </c>

</xml_diff>